<commit_message>
fix: excel and hormogch
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dope\Desktop\imp\imperial-site\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{326305B8-ABC3-40FB-B280-954F03FEA8BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{822D0B7C-5EFC-4F77-9937-9071F569DE60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2685" yWindow="2685" windowWidth="21600" windowHeight="11295" xr2:uid="{44DE746D-FE63-4989-8F77-FCA758C2B152}"/>
+    <workbookView xWindow="4470" yWindow="2370" windowWidth="21600" windowHeight="11295" xr2:uid="{44DE746D-FE63-4989-8F77-FCA758C2B152}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1066" uniqueCount="845">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="845">
   <si>
     <t>№</t>
   </si>
@@ -1913,9 +1913,6 @@
     <t>61791-26-2</t>
   </si>
   <si>
-    <t>Таннин хүчил</t>
-  </si>
-  <si>
     <t>Tannic acid</t>
   </si>
   <si>
@@ -1925,9 +1922,6 @@
     <t>1401-55-4</t>
   </si>
   <si>
-    <t>Тансгт ягаан</t>
-  </si>
-  <si>
     <t>Crystal violet</t>
   </si>
   <si>
@@ -2571,6 +2565,12 @@
   </si>
   <si>
     <t>120</t>
+  </si>
+  <si>
+    <t>Таннын хүчил</t>
+  </si>
+  <si>
+    <t>Талст ягаан</t>
   </si>
 </sst>
 </file>
@@ -3109,7 +3109,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9862B8A-AD7A-4BF2-888F-7C38CFC733CA}">
-  <dimension ref="A1:F230"/>
+  <dimension ref="A1:F229"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.5703125" customWidth="1"/>
@@ -6523,16 +6523,16 @@
         <v>172</v>
       </c>
       <c r="B171" s="6" t="s">
+        <v>843</v>
+      </c>
+      <c r="C171" s="6" t="s">
         <v>625</v>
       </c>
-      <c r="C171" s="6" t="s">
+      <c r="D171" s="6" t="s">
         <v>626</v>
       </c>
-      <c r="D171" s="6" t="s">
+      <c r="E171" s="4" t="s">
         <v>627</v>
-      </c>
-      <c r="E171" s="4" t="s">
-        <v>628</v>
       </c>
       <c r="F171" s="4" t="s">
         <v>94</v>
@@ -6543,16 +6543,16 @@
         <v>173</v>
       </c>
       <c r="B172" s="6" t="s">
+        <v>844</v>
+      </c>
+      <c r="C172" s="6" t="s">
+        <v>628</v>
+      </c>
+      <c r="D172" s="6" t="s">
         <v>629</v>
       </c>
-      <c r="C172" s="6" t="s">
+      <c r="E172" s="4" t="s">
         <v>630</v>
-      </c>
-      <c r="D172" s="6" t="s">
-        <v>631</v>
-      </c>
-      <c r="E172" s="4" t="s">
-        <v>632</v>
       </c>
       <c r="F172" s="4" t="s">
         <v>68</v>
@@ -6563,16 +6563,16 @@
         <v>174</v>
       </c>
       <c r="B173" s="6" t="s">
+        <v>631</v>
+      </c>
+      <c r="C173" s="6" t="s">
+        <v>632</v>
+      </c>
+      <c r="D173" s="6" t="s">
         <v>633</v>
       </c>
-      <c r="C173" s="6" t="s">
+      <c r="E173" s="4" t="s">
         <v>634</v>
-      </c>
-      <c r="D173" s="6" t="s">
-        <v>635</v>
-      </c>
-      <c r="E173" s="4" t="s">
-        <v>636</v>
       </c>
       <c r="F173" s="4" t="s">
         <v>111</v>
@@ -6583,16 +6583,16 @@
         <v>175</v>
       </c>
       <c r="B174" s="13" t="s">
+        <v>635</v>
+      </c>
+      <c r="C174" s="13" t="s">
+        <v>636</v>
+      </c>
+      <c r="D174" s="13" t="s">
         <v>637</v>
       </c>
-      <c r="C174" s="13" t="s">
+      <c r="E174" s="13" t="s">
         <v>638</v>
-      </c>
-      <c r="D174" s="13" t="s">
-        <v>639</v>
-      </c>
-      <c r="E174" s="13" t="s">
-        <v>640</v>
       </c>
       <c r="F174" s="13">
         <v>0.5</v>
@@ -6603,16 +6603,16 @@
         <v>176</v>
       </c>
       <c r="B175" s="8" t="s">
+        <v>639</v>
+      </c>
+      <c r="C175" s="8" t="s">
+        <v>640</v>
+      </c>
+      <c r="D175" s="8" t="s">
         <v>641</v>
       </c>
-      <c r="C175" s="8" t="s">
+      <c r="E175" s="8" t="s">
         <v>642</v>
-      </c>
-      <c r="D175" s="8" t="s">
-        <v>643</v>
-      </c>
-      <c r="E175" s="8" t="s">
-        <v>644</v>
       </c>
       <c r="F175" s="8">
         <v>500</v>
@@ -6623,16 +6623,16 @@
         <v>177</v>
       </c>
       <c r="B176" s="8" t="s">
+        <v>643</v>
+      </c>
+      <c r="C176" s="8" t="s">
+        <v>644</v>
+      </c>
+      <c r="D176" s="8" t="s">
         <v>645</v>
       </c>
-      <c r="C176" s="8" t="s">
+      <c r="E176" s="8" t="s">
         <v>646</v>
-      </c>
-      <c r="D176" s="8" t="s">
-        <v>647</v>
-      </c>
-      <c r="E176" s="8" t="s">
-        <v>648</v>
       </c>
       <c r="F176" s="8">
         <v>500</v>
@@ -6643,10 +6643,10 @@
         <v>178</v>
       </c>
       <c r="B177" s="6" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="C177" s="6" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="D177" s="6" t="s">
         <v>18</v>
@@ -6663,19 +6663,19 @@
         <v>179</v>
       </c>
       <c r="B178" s="6" t="s">
+        <v>649</v>
+      </c>
+      <c r="C178" s="6" t="s">
+        <v>650</v>
+      </c>
+      <c r="D178" s="6" t="s">
         <v>651</v>
       </c>
-      <c r="C178" s="6" t="s">
+      <c r="E178" s="4" t="s">
         <v>652</v>
       </c>
-      <c r="D178" s="6" t="s">
+      <c r="F178" s="4" t="s">
         <v>653</v>
-      </c>
-      <c r="E178" s="4" t="s">
-        <v>654</v>
-      </c>
-      <c r="F178" s="4" t="s">
-        <v>655</v>
       </c>
     </row>
     <row r="179" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -6683,19 +6683,19 @@
         <v>180</v>
       </c>
       <c r="B179" s="6" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="C179" s="6" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D179" s="6" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="E179" s="4" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="F179" s="4" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
     </row>
     <row r="180" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -6703,16 +6703,16 @@
         <v>181</v>
       </c>
       <c r="B180" s="6" t="s">
+        <v>656</v>
+      </c>
+      <c r="C180" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="D180" s="6" t="s">
         <v>658</v>
       </c>
-      <c r="C180" s="6" t="s">
+      <c r="E180" s="4" t="s">
         <v>659</v>
-      </c>
-      <c r="D180" s="6" t="s">
-        <v>660</v>
-      </c>
-      <c r="E180" s="4" t="s">
-        <v>661</v>
       </c>
       <c r="F180" s="4" t="s">
         <v>250</v>
@@ -6723,16 +6723,16 @@
         <v>182</v>
       </c>
       <c r="B181" s="6" t="s">
+        <v>660</v>
+      </c>
+      <c r="C181" s="6" t="s">
+        <v>661</v>
+      </c>
+      <c r="D181" s="6" t="s">
         <v>662</v>
       </c>
-      <c r="C181" s="6" t="s">
+      <c r="E181" s="4" t="s">
         <v>663</v>
-      </c>
-      <c r="D181" s="6" t="s">
-        <v>664</v>
-      </c>
-      <c r="E181" s="4" t="s">
-        <v>665</v>
       </c>
       <c r="F181" s="4" t="s">
         <v>15</v>
@@ -6743,16 +6743,16 @@
         <v>183</v>
       </c>
       <c r="B182" s="6" t="s">
+        <v>664</v>
+      </c>
+      <c r="C182" s="6" t="s">
+        <v>665</v>
+      </c>
+      <c r="D182" s="6" t="s">
         <v>666</v>
       </c>
-      <c r="C182" s="6" t="s">
+      <c r="E182" s="4" t="s">
         <v>667</v>
-      </c>
-      <c r="D182" s="6" t="s">
-        <v>668</v>
-      </c>
-      <c r="E182" s="4" t="s">
-        <v>669</v>
       </c>
       <c r="F182" s="4" t="s">
         <v>77</v>
@@ -6763,16 +6763,16 @@
         <v>184</v>
       </c>
       <c r="B183" s="6" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="C183" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="D183" s="6" t="s">
+        <v>669</v>
+      </c>
+      <c r="E183" s="4" t="s">
         <v>670</v>
-      </c>
-      <c r="D183" s="6" t="s">
-        <v>671</v>
-      </c>
-      <c r="E183" s="4" t="s">
-        <v>672</v>
       </c>
       <c r="F183" s="4" t="s">
         <v>15</v>
@@ -6783,16 +6783,16 @@
         <v>185</v>
       </c>
       <c r="B184" s="16" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="C184" s="16" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="D184" s="16" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="E184" s="16" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="F184" s="16">
         <v>500</v>
@@ -6803,16 +6803,16 @@
         <v>186</v>
       </c>
       <c r="B185" s="6" t="s">
+        <v>673</v>
+      </c>
+      <c r="C185" s="6" t="s">
+        <v>674</v>
+      </c>
+      <c r="D185" s="6" t="s">
         <v>675</v>
       </c>
-      <c r="C185" s="6" t="s">
+      <c r="E185" s="4" t="s">
         <v>676</v>
-      </c>
-      <c r="D185" s="6" t="s">
-        <v>677</v>
-      </c>
-      <c r="E185" s="4" t="s">
-        <v>678</v>
       </c>
       <c r="F185" s="4" t="s">
         <v>250</v>
@@ -6823,16 +6823,16 @@
         <v>187</v>
       </c>
       <c r="B186" s="6" t="s">
+        <v>677</v>
+      </c>
+      <c r="C186" s="6" t="s">
+        <v>678</v>
+      </c>
+      <c r="D186" s="6" t="s">
         <v>679</v>
       </c>
-      <c r="C186" s="6" t="s">
+      <c r="E186" s="4" t="s">
         <v>680</v>
-      </c>
-      <c r="D186" s="6" t="s">
-        <v>681</v>
-      </c>
-      <c r="E186" s="4" t="s">
-        <v>682</v>
       </c>
       <c r="F186" s="4" t="s">
         <v>10</v>
@@ -6843,16 +6843,16 @@
         <v>188</v>
       </c>
       <c r="B187" s="6" t="s">
+        <v>681</v>
+      </c>
+      <c r="C187" s="6" t="s">
+        <v>682</v>
+      </c>
+      <c r="D187" s="6" t="s">
         <v>683</v>
       </c>
-      <c r="C187" s="6" t="s">
+      <c r="E187" s="4" t="s">
         <v>684</v>
-      </c>
-      <c r="D187" s="6" t="s">
-        <v>685</v>
-      </c>
-      <c r="E187" s="4" t="s">
-        <v>686</v>
       </c>
       <c r="F187" s="4" t="s">
         <v>111</v>
@@ -6863,16 +6863,16 @@
         <v>189</v>
       </c>
       <c r="B188" s="14" t="s">
+        <v>685</v>
+      </c>
+      <c r="C188" s="13" t="s">
+        <v>686</v>
+      </c>
+      <c r="D188" s="13" t="s">
         <v>687</v>
       </c>
-      <c r="C188" s="13" t="s">
+      <c r="E188" s="13" t="s">
         <v>688</v>
-      </c>
-      <c r="D188" s="13" t="s">
-        <v>689</v>
-      </c>
-      <c r="E188" s="13" t="s">
-        <v>690</v>
       </c>
       <c r="F188" s="13">
         <v>0.5</v>
@@ -6883,16 +6883,16 @@
         <v>190</v>
       </c>
       <c r="B189" s="6" t="s">
+        <v>689</v>
+      </c>
+      <c r="C189" s="6" t="s">
+        <v>690</v>
+      </c>
+      <c r="D189" s="6" t="s">
         <v>691</v>
       </c>
-      <c r="C189" s="6" t="s">
+      <c r="E189" s="4" t="s">
         <v>692</v>
-      </c>
-      <c r="D189" s="6" t="s">
-        <v>693</v>
-      </c>
-      <c r="E189" s="4" t="s">
-        <v>694</v>
       </c>
       <c r="F189" s="4" t="s">
         <v>183</v>
@@ -6903,16 +6903,16 @@
         <v>191</v>
       </c>
       <c r="B190" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="C190" s="6" t="s">
+        <v>694</v>
+      </c>
+      <c r="D190" s="6" t="s">
         <v>695</v>
       </c>
-      <c r="C190" s="6" t="s">
+      <c r="E190" s="4" t="s">
         <v>696</v>
-      </c>
-      <c r="D190" s="6" t="s">
-        <v>697</v>
-      </c>
-      <c r="E190" s="4" t="s">
-        <v>698</v>
       </c>
       <c r="F190" s="4" t="s">
         <v>200</v>
@@ -6923,16 +6923,16 @@
         <v>192</v>
       </c>
       <c r="B191" s="8" t="s">
+        <v>697</v>
+      </c>
+      <c r="C191" s="8" t="s">
+        <v>698</v>
+      </c>
+      <c r="D191" s="8" t="s">
         <v>699</v>
       </c>
-      <c r="C191" s="8" t="s">
+      <c r="E191" s="8" t="s">
         <v>700</v>
-      </c>
-      <c r="D191" s="8" t="s">
-        <v>701</v>
-      </c>
-      <c r="E191" s="8" t="s">
-        <v>702</v>
       </c>
       <c r="F191" s="8">
         <v>500</v>
@@ -6943,16 +6943,16 @@
         <v>193</v>
       </c>
       <c r="B192" s="8" t="s">
+        <v>701</v>
+      </c>
+      <c r="C192" s="8" t="s">
+        <v>702</v>
+      </c>
+      <c r="D192" s="8" t="s">
         <v>703</v>
       </c>
-      <c r="C192" s="8" t="s">
+      <c r="E192" s="8" t="s">
         <v>704</v>
-      </c>
-      <c r="D192" s="8" t="s">
-        <v>705</v>
-      </c>
-      <c r="E192" s="8" t="s">
-        <v>706</v>
       </c>
       <c r="F192" s="8">
         <v>5</v>
@@ -6963,16 +6963,16 @@
         <v>194</v>
       </c>
       <c r="B193" s="8" t="s">
+        <v>705</v>
+      </c>
+      <c r="C193" s="8" t="s">
+        <v>706</v>
+      </c>
+      <c r="D193" s="8" t="s">
         <v>707</v>
       </c>
-      <c r="C193" s="8" t="s">
+      <c r="E193" s="8" t="s">
         <v>708</v>
-      </c>
-      <c r="D193" s="8" t="s">
-        <v>709</v>
-      </c>
-      <c r="E193" s="8" t="s">
-        <v>710</v>
       </c>
       <c r="F193" s="8">
         <v>50</v>
@@ -6983,16 +6983,16 @@
         <v>195</v>
       </c>
       <c r="B194" s="8" t="s">
+        <v>709</v>
+      </c>
+      <c r="C194" s="8" t="s">
+        <v>710</v>
+      </c>
+      <c r="D194" s="8" t="s">
         <v>711</v>
       </c>
-      <c r="C194" s="8" t="s">
+      <c r="E194" s="8" t="s">
         <v>712</v>
-      </c>
-      <c r="D194" s="8" t="s">
-        <v>713</v>
-      </c>
-      <c r="E194" s="8" t="s">
-        <v>714</v>
       </c>
       <c r="F194" s="8">
         <v>100</v>
@@ -7003,16 +7003,16 @@
         <v>196</v>
       </c>
       <c r="B195" s="8" t="s">
+        <v>713</v>
+      </c>
+      <c r="C195" s="17" t="s">
+        <v>714</v>
+      </c>
+      <c r="D195" s="18" t="s">
         <v>715</v>
       </c>
-      <c r="C195" s="17" t="s">
+      <c r="E195" s="16" t="s">
         <v>716</v>
-      </c>
-      <c r="D195" s="18" t="s">
-        <v>717</v>
-      </c>
-      <c r="E195" s="16" t="s">
-        <v>718</v>
       </c>
       <c r="F195" s="16">
         <v>1000</v>
@@ -7023,14 +7023,14 @@
         <v>197</v>
       </c>
       <c r="B196" s="16" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="C196" s="16" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="D196" s="16"/>
       <c r="E196" s="16" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="F196" s="19">
         <v>1000</v>
@@ -7041,16 +7041,16 @@
         <v>198</v>
       </c>
       <c r="B197" s="6" t="s">
+        <v>720</v>
+      </c>
+      <c r="C197" s="6" t="s">
+        <v>721</v>
+      </c>
+      <c r="D197" s="6" t="s">
         <v>722</v>
       </c>
-      <c r="C197" s="6" t="s">
+      <c r="E197" s="4" t="s">
         <v>723</v>
-      </c>
-      <c r="D197" s="6" t="s">
-        <v>724</v>
-      </c>
-      <c r="E197" s="4" t="s">
-        <v>725</v>
       </c>
       <c r="F197" s="4" t="s">
         <v>68</v>
@@ -7061,16 +7061,16 @@
         <v>199</v>
       </c>
       <c r="B198" s="6" t="s">
+        <v>724</v>
+      </c>
+      <c r="C198" s="6" t="s">
+        <v>725</v>
+      </c>
+      <c r="D198" s="6" t="s">
         <v>726</v>
       </c>
-      <c r="C198" s="6" t="s">
+      <c r="E198" s="4" t="s">
         <v>727</v>
-      </c>
-      <c r="D198" s="6" t="s">
-        <v>728</v>
-      </c>
-      <c r="E198" s="4" t="s">
-        <v>729</v>
       </c>
       <c r="F198" s="4" t="s">
         <v>68</v>
@@ -7081,16 +7081,16 @@
         <v>200</v>
       </c>
       <c r="B199" s="8" t="s">
+        <v>728</v>
+      </c>
+      <c r="C199" s="8" t="s">
+        <v>729</v>
+      </c>
+      <c r="D199" s="8" t="s">
         <v>730</v>
       </c>
-      <c r="C199" s="8" t="s">
+      <c r="E199" s="8" t="s">
         <v>731</v>
-      </c>
-      <c r="D199" s="8" t="s">
-        <v>732</v>
-      </c>
-      <c r="E199" s="8" t="s">
-        <v>733</v>
       </c>
       <c r="F199" s="8">
         <v>200</v>
@@ -7101,16 +7101,16 @@
         <v>201</v>
       </c>
       <c r="B200" s="6" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="C200" s="6" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="D200" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E200" s="4" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="F200" s="4" t="s">
         <v>250</v>
@@ -7121,16 +7121,16 @@
         <v>202</v>
       </c>
       <c r="B201" s="8" t="s">
+        <v>735</v>
+      </c>
+      <c r="C201" s="8" t="s">
+        <v>736</v>
+      </c>
+      <c r="D201" s="8" t="s">
         <v>737</v>
       </c>
-      <c r="C201" s="8" t="s">
+      <c r="E201" s="8" t="s">
         <v>738</v>
-      </c>
-      <c r="D201" s="8" t="s">
-        <v>739</v>
-      </c>
-      <c r="E201" s="8" t="s">
-        <v>740</v>
       </c>
       <c r="F201" s="8">
         <v>500</v>
@@ -7141,16 +7141,16 @@
         <v>203</v>
       </c>
       <c r="B202" s="6" t="s">
+        <v>739</v>
+      </c>
+      <c r="C202" s="6" t="s">
+        <v>740</v>
+      </c>
+      <c r="D202" s="6" t="s">
         <v>741</v>
       </c>
-      <c r="C202" s="6" t="s">
+      <c r="E202" s="4" t="s">
         <v>742</v>
-      </c>
-      <c r="D202" s="6" t="s">
-        <v>743</v>
-      </c>
-      <c r="E202" s="4" t="s">
-        <v>744</v>
       </c>
       <c r="F202" s="4" t="s">
         <v>15</v>
@@ -7161,16 +7161,16 @@
         <v>204</v>
       </c>
       <c r="B203" s="6" t="s">
+        <v>743</v>
+      </c>
+      <c r="C203" s="6" t="s">
+        <v>744</v>
+      </c>
+      <c r="D203" s="6" t="s">
         <v>745</v>
       </c>
-      <c r="C203" s="6" t="s">
+      <c r="E203" s="4" t="s">
         <v>746</v>
-      </c>
-      <c r="D203" s="6" t="s">
-        <v>747</v>
-      </c>
-      <c r="E203" s="4" t="s">
-        <v>748</v>
       </c>
       <c r="F203" s="4" t="s">
         <v>94</v>
@@ -7178,542 +7178,522 @@
     </row>
     <row r="204" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A204" s="4">
-        <v>205</v>
-      </c>
-      <c r="B204" s="16" t="s">
-        <v>745</v>
-      </c>
-      <c r="C204" s="16" t="s">
-        <v>746</v>
-      </c>
-      <c r="D204" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="B204" s="6" t="s">
         <v>747</v>
       </c>
-      <c r="E204" s="16" t="s">
+      <c r="C204" s="6" t="s">
         <v>748</v>
       </c>
-      <c r="F204" s="16">
-        <v>500</v>
+      <c r="D204" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E204" s="4" t="s">
+        <v>749</v>
+      </c>
+      <c r="F204" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="205" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A205" s="4">
-        <v>206</v>
-      </c>
-      <c r="B205" s="6" t="s">
-        <v>749</v>
-      </c>
-      <c r="C205" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="B205" s="8" t="s">
         <v>750</v>
       </c>
-      <c r="D205" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E205" s="4" t="s">
+      <c r="C205" s="8" t="s">
         <v>751</v>
       </c>
-      <c r="F205" s="4" t="s">
-        <v>10</v>
+      <c r="D205" s="8" t="s">
+        <v>752</v>
+      </c>
+      <c r="E205" s="8" t="s">
+        <v>753</v>
+      </c>
+      <c r="F205" s="8">
+        <v>500</v>
       </c>
     </row>
     <row r="206" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A206" s="4">
-        <v>207</v>
-      </c>
-      <c r="B206" s="8" t="s">
-        <v>752</v>
-      </c>
-      <c r="C206" s="8" t="s">
-        <v>753</v>
-      </c>
-      <c r="D206" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="B206" s="6" t="s">
         <v>754</v>
       </c>
-      <c r="E206" s="8" t="s">
+      <c r="C206" s="6" t="s">
         <v>755</v>
       </c>
-      <c r="F206" s="8">
-        <v>500</v>
+      <c r="D206" s="6" t="s">
+        <v>756</v>
+      </c>
+      <c r="E206" s="4" t="s">
+        <v>757</v>
+      </c>
+      <c r="F206" s="4" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="207" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A207" s="4">
-        <v>208</v>
-      </c>
-      <c r="B207" s="6" t="s">
-        <v>756</v>
-      </c>
-      <c r="C207" s="6" t="s">
-        <v>757</v>
-      </c>
-      <c r="D207" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="B207" s="8" t="s">
         <v>758</v>
       </c>
-      <c r="E207" s="4" t="s">
+      <c r="C207" s="16" t="s">
         <v>759</v>
       </c>
-      <c r="F207" s="4" t="s">
-        <v>94</v>
+      <c r="D207" s="8" t="s">
+        <v>468</v>
+      </c>
+      <c r="E207" s="8" t="s">
+        <v>469</v>
+      </c>
+      <c r="F207" s="16">
+        <v>1000</v>
       </c>
     </row>
     <row r="208" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A208" s="4">
-        <v>209</v>
-      </c>
-      <c r="B208" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="B208" s="6" t="s">
         <v>760</v>
       </c>
-      <c r="C208" s="16" t="s">
+      <c r="C208" s="6" t="s">
         <v>761</v>
       </c>
-      <c r="D208" s="8" t="s">
-        <v>468</v>
-      </c>
-      <c r="E208" s="8" t="s">
-        <v>469</v>
-      </c>
-      <c r="F208" s="16">
-        <v>1000</v>
+      <c r="D208" s="6" t="s">
+        <v>762</v>
+      </c>
+      <c r="E208" s="4" t="s">
+        <v>763</v>
+      </c>
+      <c r="F208" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="209" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A209" s="4">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B209" s="6" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="C209" s="6" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="D209" s="6" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="E209" s="4" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="F209" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="210" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A210" s="4">
-        <v>211</v>
-      </c>
-      <c r="B210" s="6" t="s">
-        <v>766</v>
-      </c>
-      <c r="C210" s="6" t="s">
-        <v>767</v>
-      </c>
-      <c r="D210" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="B210" s="8" t="s">
         <v>768</v>
       </c>
-      <c r="E210" s="4" t="s">
+      <c r="C210" s="8" t="s">
+        <v>459</v>
+      </c>
+      <c r="D210" s="8" t="s">
         <v>769</v>
       </c>
-      <c r="F210" s="4" t="s">
-        <v>250</v>
+      <c r="E210" s="8" t="s">
+        <v>770</v>
+      </c>
+      <c r="F210" s="8">
+        <v>100</v>
       </c>
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A211" s="4">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B211" s="8" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="C211" s="8" t="s">
-        <v>459</v>
+        <v>772</v>
       </c>
       <c r="D211" s="8" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="E211" s="8" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="F211" s="8">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="212" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A212" s="4">
-        <v>213</v>
-      </c>
-      <c r="B212" s="8" t="s">
-        <v>773</v>
-      </c>
-      <c r="C212" s="8" t="s">
-        <v>774</v>
-      </c>
-      <c r="D212" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="B212" s="6" t="s">
         <v>775</v>
       </c>
-      <c r="E212" s="8" t="s">
+      <c r="C212" s="6" t="s">
         <v>776</v>
       </c>
-      <c r="F212" s="8">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="213" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="D212" s="6" t="s">
+        <v>777</v>
+      </c>
+      <c r="E212" s="4" t="s">
+        <v>778</v>
+      </c>
+      <c r="F212" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A213" s="4">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B213" s="6" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
       <c r="C213" s="6" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="D213" s="6" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="E213" s="4" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="F213" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="214" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A214" s="4">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B214" s="6" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="C214" s="6" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="D214" s="6" t="s">
-        <v>783</v>
+        <v>18</v>
       </c>
       <c r="E214" s="4" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="F214" s="4" t="s">
-        <v>94</v>
+        <v>10</v>
       </c>
     </row>
     <row r="215" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A215" s="4">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B215" s="6" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="C215" s="6" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="D215" s="6" t="s">
-        <v>18</v>
+        <v>788</v>
       </c>
       <c r="E215" s="4" t="s">
-        <v>787</v>
+        <v>789</v>
       </c>
       <c r="F215" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="216" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A216" s="4">
+        <v>218</v>
+      </c>
+      <c r="B216" s="6" t="s">
+        <v>790</v>
+      </c>
+      <c r="C216" s="6" t="s">
+        <v>791</v>
+      </c>
+      <c r="D216" s="6" t="s">
+        <v>792</v>
+      </c>
+      <c r="E216" s="4" t="s">
+        <v>793</v>
+      </c>
+      <c r="F216" s="4" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="216" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A216" s="4">
-        <v>217</v>
-      </c>
-      <c r="B216" s="6" t="s">
-        <v>788</v>
-      </c>
-      <c r="C216" s="6" t="s">
-        <v>789</v>
-      </c>
-      <c r="D216" s="6" t="s">
-        <v>790</v>
-      </c>
-      <c r="E216" s="4" t="s">
-        <v>791</v>
-      </c>
-      <c r="F216" s="4" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="217" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A217" s="4">
-        <v>218</v>
-      </c>
-      <c r="B217" s="6" t="s">
-        <v>792</v>
-      </c>
-      <c r="C217" s="6" t="s">
-        <v>793</v>
-      </c>
-      <c r="D217" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="B217" s="8" t="s">
         <v>794</v>
       </c>
-      <c r="E217" s="4" t="s">
+      <c r="C217" s="8" t="s">
         <v>795</v>
       </c>
-      <c r="F217" s="4" t="s">
-        <v>10</v>
+      <c r="D217" s="8" t="s">
+        <v>796</v>
+      </c>
+      <c r="E217" s="8" t="s">
+        <v>797</v>
+      </c>
+      <c r="F217" s="8">
+        <v>100</v>
       </c>
     </row>
     <row r="218" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A218" s="4">
-        <v>219</v>
-      </c>
-      <c r="B218" s="8" t="s">
-        <v>796</v>
-      </c>
-      <c r="C218" s="8" t="s">
-        <v>797</v>
-      </c>
-      <c r="D218" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="B218" s="6" t="s">
         <v>798</v>
       </c>
-      <c r="E218" s="8" t="s">
+      <c r="C218" s="6" t="s">
         <v>799</v>
       </c>
-      <c r="F218" s="8">
-        <v>100</v>
+      <c r="D218" s="6" t="s">
+        <v>800</v>
+      </c>
+      <c r="E218" s="4" t="s">
+        <v>801</v>
+      </c>
+      <c r="F218" s="4" t="s">
+        <v>802</v>
       </c>
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A219" s="4">
-        <v>220</v>
-      </c>
-      <c r="B219" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="B219" s="8" t="s">
+        <v>798</v>
+      </c>
+      <c r="C219" s="8" t="s">
+        <v>799</v>
+      </c>
+      <c r="D219" s="8" t="s">
         <v>800</v>
       </c>
-      <c r="C219" s="6" t="s">
+      <c r="E219" s="8" t="s">
         <v>801</v>
       </c>
-      <c r="D219" s="6" t="s">
-        <v>802</v>
-      </c>
-      <c r="E219" s="4" t="s">
+      <c r="F219" s="20">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="220" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A220" s="4">
+        <v>222</v>
+      </c>
+      <c r="B220" s="6" t="s">
         <v>803</v>
       </c>
-      <c r="F219" s="4" t="s">
+      <c r="C220" s="6" t="s">
         <v>804</v>
       </c>
-    </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A220" s="4">
-        <v>221</v>
-      </c>
-      <c r="B220" s="8" t="s">
-        <v>800</v>
-      </c>
-      <c r="C220" s="8" t="s">
-        <v>801</v>
-      </c>
-      <c r="D220" s="8" t="s">
-        <v>802</v>
-      </c>
-      <c r="E220" s="8" t="s">
-        <v>803</v>
-      </c>
-      <c r="F220" s="20">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="221" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="D220" s="6" t="s">
+        <v>805</v>
+      </c>
+      <c r="E220" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="F220" s="4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="221" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A221" s="4">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B221" s="6" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="C221" s="6" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="D221" s="6" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="E221" s="4" t="s">
-        <v>555</v>
+        <v>809</v>
       </c>
       <c r="F221" s="4" t="s">
-        <v>147</v>
+        <v>94</v>
       </c>
     </row>
     <row r="222" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A222" s="4">
-        <v>223</v>
-      </c>
-      <c r="B222" s="6" t="s">
-        <v>808</v>
-      </c>
-      <c r="C222" s="6" t="s">
-        <v>809</v>
-      </c>
-      <c r="D222" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="B222" s="8" t="s">
         <v>810</v>
       </c>
-      <c r="E222" s="4" t="s">
+      <c r="C222" s="8" t="s">
         <v>811</v>
       </c>
-      <c r="F222" s="4" t="s">
-        <v>94</v>
+      <c r="D222" s="8" t="s">
+        <v>812</v>
+      </c>
+      <c r="E222" s="8" t="s">
+        <v>813</v>
+      </c>
+      <c r="F222" s="8">
+        <v>200</v>
       </c>
     </row>
     <row r="223" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A223" s="4">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B223" s="8" t="s">
-        <v>812</v>
+        <v>814</v>
       </c>
       <c r="C223" s="8" t="s">
-        <v>813</v>
+        <v>815</v>
       </c>
       <c r="D223" s="8" t="s">
-        <v>814</v>
+        <v>816</v>
       </c>
       <c r="E223" s="8" t="s">
-        <v>815</v>
+        <v>817</v>
       </c>
       <c r="F223" s="8">
-        <v>200</v>
+        <v>100</v>
       </c>
     </row>
     <row r="224" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A224" s="4">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B224" s="8" t="s">
-        <v>816</v>
+        <v>818</v>
       </c>
       <c r="C224" s="8" t="s">
-        <v>817</v>
+        <v>819</v>
       </c>
       <c r="D224" s="8" t="s">
-        <v>818</v>
+        <v>820</v>
       </c>
       <c r="E224" s="8" t="s">
-        <v>819</v>
+        <v>821</v>
       </c>
       <c r="F224" s="8">
-        <v>100</v>
+        <v>200</v>
       </c>
     </row>
     <row r="225" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A225" s="4">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B225" s="8" t="s">
-        <v>820</v>
-      </c>
-      <c r="C225" s="8" t="s">
-        <v>821</v>
-      </c>
-      <c r="D225" s="8" t="s">
         <v>822</v>
       </c>
-      <c r="E225" s="8" t="s">
+      <c r="C225" s="13" t="s">
         <v>823</v>
       </c>
-      <c r="F225" s="8">
-        <v>200</v>
+      <c r="D225" s="13" t="s">
+        <v>824</v>
+      </c>
+      <c r="E225" s="13" t="s">
+        <v>825</v>
+      </c>
+      <c r="F225" s="13">
+        <v>1</v>
       </c>
     </row>
     <row r="226" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A226" s="4">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B226" s="8" t="s">
-        <v>824</v>
-      </c>
-      <c r="C226" s="13" t="s">
-        <v>825</v>
-      </c>
-      <c r="D226" s="13" t="s">
         <v>826</v>
       </c>
-      <c r="E226" s="13" t="s">
+      <c r="C226" s="8" t="s">
         <v>827</v>
       </c>
-      <c r="F226" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D226" s="8" t="s">
+        <v>828</v>
+      </c>
+      <c r="E226" s="8" t="s">
+        <v>829</v>
+      </c>
+      <c r="F226" s="16">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="227" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A227" s="4">
-        <v>228</v>
-      </c>
-      <c r="B227" s="8" t="s">
-        <v>828</v>
-      </c>
-      <c r="C227" s="8" t="s">
-        <v>829</v>
-      </c>
-      <c r="D227" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="B227" s="6" t="s">
         <v>830</v>
       </c>
-      <c r="E227" s="8" t="s">
+      <c r="C227" s="6" t="s">
         <v>831</v>
       </c>
-      <c r="F227" s="16">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="228" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="D227" s="6" t="s">
+        <v>832</v>
+      </c>
+      <c r="E227" s="4" t="s">
+        <v>833</v>
+      </c>
+      <c r="F227" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A228" s="4">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B228" s="6" t="s">
-        <v>832</v>
+        <v>834</v>
       </c>
       <c r="C228" s="6" t="s">
-        <v>833</v>
+        <v>835</v>
       </c>
       <c r="D228" s="6" t="s">
-        <v>834</v>
+        <v>836</v>
       </c>
       <c r="E228" s="4" t="s">
-        <v>835</v>
+        <v>837</v>
       </c>
       <c r="F228" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="229" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A229" s="4">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B229" s="6" t="s">
-        <v>836</v>
+        <v>838</v>
       </c>
       <c r="C229" s="6" t="s">
-        <v>837</v>
+        <v>839</v>
       </c>
       <c r="D229" s="6" t="s">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="E229" s="4" t="s">
-        <v>839</v>
+        <v>841</v>
       </c>
       <c r="F229" s="4" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="230" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A230" s="4">
-        <v>231</v>
-      </c>
-      <c r="B230" s="6" t="s">
-        <v>840</v>
-      </c>
-      <c r="C230" s="6" t="s">
-        <v>841</v>
-      </c>
-      <c r="D230" s="6" t="s">
         <v>842</v>
-      </c>
-      <c r="E230" s="4" t="s">
-        <v>843</v>
-      </c>
-      <c r="F230" s="4" t="s">
-        <v>844</v>
       </c>
     </row>
   </sheetData>

</xml_diff>